<commit_message>
Historia de usuario v15: tercera ronda con veredicto de salida a producción
- Historia_de_usuario_Rehavid_v15.xlsx: historia por épicas (0 a 9 +
  transversal + veredicto), hoja «Flujo del app» con el diagrama, una
  pestaña por cargo que cierra sus hallazgos de la segunda ronda
  (CORREGIDO EN v15 / PENDIENTE con prioridad a confirmar), revisión de
  su base de alimentación, y tabla de decisión de salida a producción
  con desplegable (Sí · Con ajustes menores · No).
- Bases regeneradas con las instrucciones de la v15 (bases_v15.py).
- Generadores versionados: contenido_v15, diagrama_v15, construir_v15.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J7RCgg76gjh3iFAK7tfLBo
</commit_message>
<xml_diff>
--- a/entregables/gestion-proyectos/bases/Base_BI.xlsx
+++ b/entregables/gestion-proyectos/bases/Base_BI.xlsx
@@ -618,14 +618,14 @@
     <row r="17">
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Abra la aplicación → módulo 09 Bases y auditoría → tarjeta «Bases de alimentación (Excel)» →</t>
+          <t>Abra la aplicación → barra lateral → Bases y auditoría → «Cargar base de alimentación (Excel)» →</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>«Subir base de alimentación» → elija este archivo. La carga NO borra lo existente: crea lo nuevo y</t>
+          <t>elija este archivo (también desde la pestaña Guía, botón «Cargar una base ahora»). La carga NO borra lo existente: crea lo nuevo y</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Versión final: historia de usuario v16, documento del flujo y bases con responsable
- Historia_de_usuario_Rehavid_v16.xlsx: ronda de aceptación — cada cargo
  verifica sus hallazgos de la 3.ª ronda aplicados, valida el modelo de
  administradores y firma la decisión de salida a producción.
- Flujo_del_app_Rehavid.pdf: portada, diagrama v16 del flujo completo
  (qué entra, qué opera, qué sale), módulos con capturas, gestión
  diaria y la tabla del modelo de permisos.
- Bases v16: columna «responsable» en Productos (elegir cargo desde el
  Excel, p. ej. Gestor de Datos 1 o 2) e instrucciones de carga por
  administradores; ejemplo con Gestor de Datos 2.
- Generadores versionados v16 en herramientas/; READMEs finales.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J7RCgg76gjh3iFAK7tfLBo
</commit_message>
<xml_diff>
--- a/entregables/gestion-proyectos/bases/Base_BI.xlsx
+++ b/entregables/gestion-proyectos/bases/Base_BI.xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B27"/>
+  <dimension ref="B2:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -618,14 +618,14 @@
     <row r="17">
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Abra la aplicación → barra lateral → Bases y auditoría → «Cargar base de alimentación (Excel)» →</t>
+          <t>La carga la hace un ADMINISTRADOR (CEO, Gerente, Director de Proyectos o Jefe de Operaciones):</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>elija este archivo (también desde la pestaña Guía, botón «Cargar una base ahora»). La carga NO borra lo existente: crea lo nuevo y</t>
+          <t>barra lateral → Bases y auditoría → «Cargar base de alimentación (Excel)» → elija este archivo. La carga NO borra lo existente: crea lo nuevo y</t>
         </is>
       </c>
     </row>
@@ -649,40 +649,47 @@
     <row r="22">
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>· El cargo responsable de cada producto lo asigna el motor según la categoría (no se escribe en la base):</t>
+          <t>· El cargo responsable lo asigna el motor según la categoría, salvo que la columna «responsable» traiga</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Medición objetiva → Director de Proyectos · Tablero BI → Gestor de Datos 1 · Diseño → Diseñador ·</t>
+          <t xml:space="preserve">  uno de los ocho cargos (sirve, por ejemplo, para elegir entre Gestor de Datos 1 y 2):</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cápsulas → Supervisor Contactabilidad · Otro → coordinación del tipo.</t>
+          <t xml:space="preserve">  Medición objetiva → Director de Proyectos · Tablero BI → Gestor de Datos 1 · Diseño → Diseñador ·</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>· Los usuarios de la aplicación son los ocho cargos: CEO, Gerente, Director de Proyectos, Jefe de Operaciones, Supervisor Contactabilidad, Gestor de Datos 1, Gestor de Datos 2, Diseñador.</t>
+          <t xml:space="preserve">  Cápsulas → Supervisor Contactabilidad · Otro → coordinación del tipo.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>· Empresas, PPR y órdenes que no existan se crean en el catálogo automáticamente.</t>
+          <t>· Los usuarios de la aplicación son los ocho cargos: CEO, Gerente, Director de Proyectos, Jefe de Operaciones, Supervisor Contactabilidad, Gestor de Datos 1, Gestor de Datos 2, Diseñador.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>· Empresas, PPR y órdenes que no existan se crean en el catálogo automáticamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>· El seguimiento se registra como novedades en la bitácora del producto, con su tipo y su fecha.</t>
         </is>
@@ -1330,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:O36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1347,6 +1354,7 @@
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1368,6 +1376,7 @@
       <c r="L1" s="5" t="n"/>
       <c r="M1" s="5" t="n"/>
       <c r="N1" s="5" t="n"/>
+      <c r="O1" s="5" t="n"/>
     </row>
     <row r="2" ht="3" customHeight="1">
       <c r="A2" s="6" t="n"/>
@@ -1384,6 +1393,7 @@
       <c r="L2" s="6" t="n"/>
       <c r="M2" s="6" t="n"/>
       <c r="N2" s="6" t="n"/>
+      <c r="O2" s="6" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
@@ -1456,6 +1466,11 @@
           <t>notas</t>
         </is>
       </c>
+      <c r="O3" s="7" t="inlineStr">
+        <is>
+          <t>responsable</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -1526,6 +1541,11 @@
       <c r="N4" s="8" t="inlineStr">
         <is>
           <t>Opcional.</t>
+        </is>
+      </c>
+      <c r="O4" s="8" t="inlineStr">
+        <is>
+          <t>Opcional. Uno de los ocho cargos; si va vacío, asigna el motor.</t>
         </is>
       </c>
     </row>
@@ -1616,6 +1636,11 @@
       <c r="L6" s="12" t="inlineStr"/>
       <c r="M6" s="12" t="inlineStr"/>
       <c r="N6" s="12" t="inlineStr"/>
+      <c r="O6" s="12" t="inlineStr">
+        <is>
+          <t>Gestor de Datos 2</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="n"/>
@@ -1632,6 +1657,7 @@
       <c r="L7" s="11" t="n"/>
       <c r="M7" s="11" t="n"/>
       <c r="N7" s="11" t="n"/>
+      <c r="O7" s="11" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="n"/>
@@ -1648,6 +1674,7 @@
       <c r="L8" s="10" t="n"/>
       <c r="M8" s="10" t="n"/>
       <c r="N8" s="10" t="n"/>
+      <c r="O8" s="10" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="11" t="n"/>
@@ -1664,6 +1691,7 @@
       <c r="L9" s="11" t="n"/>
       <c r="M9" s="11" t="n"/>
       <c r="N9" s="11" t="n"/>
+      <c r="O9" s="11" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="n"/>
@@ -1680,6 +1708,7 @@
       <c r="L10" s="10" t="n"/>
       <c r="M10" s="10" t="n"/>
       <c r="N10" s="10" t="n"/>
+      <c r="O10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="11" t="n"/>
@@ -1696,6 +1725,7 @@
       <c r="L11" s="11" t="n"/>
       <c r="M11" s="11" t="n"/>
       <c r="N11" s="11" t="n"/>
+      <c r="O11" s="11" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="n"/>
@@ -1712,6 +1742,7 @@
       <c r="L12" s="10" t="n"/>
       <c r="M12" s="10" t="n"/>
       <c r="N12" s="10" t="n"/>
+      <c r="O12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="11" t="n"/>
@@ -1728,6 +1759,7 @@
       <c r="L13" s="11" t="n"/>
       <c r="M13" s="11" t="n"/>
       <c r="N13" s="11" t="n"/>
+      <c r="O13" s="11" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="n"/>
@@ -1744,6 +1776,7 @@
       <c r="L14" s="10" t="n"/>
       <c r="M14" s="10" t="n"/>
       <c r="N14" s="10" t="n"/>
+      <c r="O14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="11" t="n"/>
@@ -1760,6 +1793,7 @@
       <c r="L15" s="11" t="n"/>
       <c r="M15" s="11" t="n"/>
       <c r="N15" s="11" t="n"/>
+      <c r="O15" s="11" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n"/>
@@ -1776,6 +1810,7 @@
       <c r="L16" s="10" t="n"/>
       <c r="M16" s="10" t="n"/>
       <c r="N16" s="10" t="n"/>
+      <c r="O16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="11" t="n"/>
@@ -1792,6 +1827,7 @@
       <c r="L17" s="11" t="n"/>
       <c r="M17" s="11" t="n"/>
       <c r="N17" s="11" t="n"/>
+      <c r="O17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n"/>
@@ -1808,6 +1844,7 @@
       <c r="L18" s="10" t="n"/>
       <c r="M18" s="10" t="n"/>
       <c r="N18" s="10" t="n"/>
+      <c r="O18" s="10" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="11" t="n"/>
@@ -1824,6 +1861,7 @@
       <c r="L19" s="11" t="n"/>
       <c r="M19" s="11" t="n"/>
       <c r="N19" s="11" t="n"/>
+      <c r="O19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n"/>
@@ -1840,6 +1878,7 @@
       <c r="L20" s="10" t="n"/>
       <c r="M20" s="10" t="n"/>
       <c r="N20" s="10" t="n"/>
+      <c r="O20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="11" t="n"/>
@@ -1856,6 +1895,7 @@
       <c r="L21" s="11" t="n"/>
       <c r="M21" s="11" t="n"/>
       <c r="N21" s="11" t="n"/>
+      <c r="O21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n"/>
@@ -1872,6 +1912,7 @@
       <c r="L22" s="10" t="n"/>
       <c r="M22" s="10" t="n"/>
       <c r="N22" s="10" t="n"/>
+      <c r="O22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="11" t="n"/>
@@ -1888,6 +1929,7 @@
       <c r="L23" s="11" t="n"/>
       <c r="M23" s="11" t="n"/>
       <c r="N23" s="11" t="n"/>
+      <c r="O23" s="11" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n"/>
@@ -1904,6 +1946,7 @@
       <c r="L24" s="10" t="n"/>
       <c r="M24" s="10" t="n"/>
       <c r="N24" s="10" t="n"/>
+      <c r="O24" s="10" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="11" t="n"/>
@@ -1920,6 +1963,7 @@
       <c r="L25" s="11" t="n"/>
       <c r="M25" s="11" t="n"/>
       <c r="N25" s="11" t="n"/>
+      <c r="O25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n"/>
@@ -1936,6 +1980,7 @@
       <c r="L26" s="10" t="n"/>
       <c r="M26" s="10" t="n"/>
       <c r="N26" s="10" t="n"/>
+      <c r="O26" s="10" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="11" t="n"/>
@@ -1952,6 +1997,7 @@
       <c r="L27" s="11" t="n"/>
       <c r="M27" s="11" t="n"/>
       <c r="N27" s="11" t="n"/>
+      <c r="O27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n"/>
@@ -1968,6 +2014,7 @@
       <c r="L28" s="10" t="n"/>
       <c r="M28" s="10" t="n"/>
       <c r="N28" s="10" t="n"/>
+      <c r="O28" s="10" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="11" t="n"/>
@@ -1984,6 +2031,7 @@
       <c r="L29" s="11" t="n"/>
       <c r="M29" s="11" t="n"/>
       <c r="N29" s="11" t="n"/>
+      <c r="O29" s="11" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n"/>
@@ -2000,6 +2048,7 @@
       <c r="L30" s="10" t="n"/>
       <c r="M30" s="10" t="n"/>
       <c r="N30" s="10" t="n"/>
+      <c r="O30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="11" t="n"/>
@@ -2016,6 +2065,7 @@
       <c r="L31" s="11" t="n"/>
       <c r="M31" s="11" t="n"/>
       <c r="N31" s="11" t="n"/>
+      <c r="O31" s="11" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n"/>
@@ -2032,6 +2082,7 @@
       <c r="L32" s="10" t="n"/>
       <c r="M32" s="10" t="n"/>
       <c r="N32" s="10" t="n"/>
+      <c r="O32" s="10" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="11" t="n"/>
@@ -2048,6 +2099,7 @@
       <c r="L33" s="11" t="n"/>
       <c r="M33" s="11" t="n"/>
       <c r="N33" s="11" t="n"/>
+      <c r="O33" s="11" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="n"/>
@@ -2064,6 +2116,7 @@
       <c r="L34" s="10" t="n"/>
       <c r="M34" s="10" t="n"/>
       <c r="N34" s="10" t="n"/>
+      <c r="O34" s="10" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="11" t="n"/>
@@ -2080,6 +2133,7 @@
       <c r="L35" s="11" t="n"/>
       <c r="M35" s="11" t="n"/>
       <c r="N35" s="11" t="n"/>
+      <c r="O35" s="11" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="n"/>
@@ -2096,11 +2150,12 @@
       <c r="L36" s="10" t="n"/>
       <c r="M36" s="10" t="n"/>
       <c r="N36" s="10" t="n"/>
+      <c r="O36" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:O2"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="C5:C36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
Bases v16: la instrucción de carga referencia el módulo Perfiles y accesos
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J7RCgg76gjh3iFAK7tfLBo
</commit_message>
<xml_diff>
--- a/entregables/gestion-proyectos/bases/Base_BI.xlsx
+++ b/entregables/gestion-proyectos/bases/Base_BI.xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B28"/>
+  <dimension ref="B2:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -618,78 +618,85 @@
     <row r="17">
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>La carga la hace un ADMINISTRADOR (CEO, Gerente, Director de Proyectos o Jefe de Operaciones):</t>
+          <t>La carga la hace un ADMINISTRADOR (por defecto CEO, Gerente, Director de Proyectos y Jefe de</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>barra lateral → Bases y auditoría → «Cargar base de alimentación (Excel)» → elija este archivo. La carga NO borra lo existente: crea lo nuevo y</t>
+          <t>Operaciones; el perfil se asigna en la app: Parametrización → Perfiles y accesos):</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="2" t="inlineStr">
         <is>
+          <t>barra lateral → Bases y auditoría → «Cargar base de alimentación (Excel)» → elija este archivo. La carga NO borra lo existente: crea lo nuevo y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="2" t="inlineStr">
+        <is>
           <t>actualiza lo que coincida por código de proyecto y nombre de producto, y muestra un resumen de lo cargado.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="2" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>REGLAS QUE APLICA LA CARGA</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>· El cargo responsable lo asigna el motor según la categoría, salvo que la columna «responsable» traiga</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  uno de los ocho cargos (sirve, por ejemplo, para elegir entre Gestor de Datos 1 y 2):</t>
+          <t>· El cargo responsable lo asigna el motor según la categoría, salvo que la columna «responsable» traiga</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Medición objetiva → Director de Proyectos · Tablero BI → Gestor de Datos 1 · Diseño → Diseñador ·</t>
+          <t xml:space="preserve">  uno de los ocho cargos (sirve, por ejemplo, para elegir entre Gestor de Datos 1 y 2):</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cápsulas → Supervisor Contactabilidad · Otro → coordinación del tipo.</t>
+          <t xml:space="preserve">  Medición objetiva → Director de Proyectos · Tablero BI → Gestor de Datos 1 · Diseño → Diseñador ·</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>· Los usuarios de la aplicación son los ocho cargos: CEO, Gerente, Director de Proyectos, Jefe de Operaciones, Supervisor Contactabilidad, Gestor de Datos 1, Gestor de Datos 2, Diseñador.</t>
+          <t xml:space="preserve">  Cápsulas → Supervisor Contactabilidad · Otro → coordinación del tipo.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>· Empresas, PPR y órdenes que no existan se crean en el catálogo automáticamente.</t>
+          <t>· Los usuarios de la aplicación son los ocho cargos: CEO, Gerente, Director de Proyectos, Jefe de Operaciones, Supervisor Contactabilidad, Gestor de Datos 1, Gestor de Datos 2, Diseñador.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>· Empresas, PPR y órdenes que no existan se crean en el catálogo automáticamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>· El seguimiento se registra como novedades en la bitácora del producto, con su tipo y su fecha.</t>
         </is>

</xml_diff>